<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-04 Le collier de maman
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-04.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-04.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, boîte à couture, rideau de dentelle</t>
+          <t>salon, boîte à couture, rideau de dentelle, pelote de laine</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut enfiler un collier de perles de bois pour maman. Elle propose. Victorino regarde, dit plus tard, dit non pour une perle. Une perle se cache dans la dentelle. Nina accepte. Maman met le collier. Il tape tout doux.</t>
+          <t>Un carré de soleil perce le rideau de dentelle. Sur le couvercle, un éclat de couvercle brille. Nina veut un collier pour maman, maintenant. Elle pousse le fil trop vite : Victorino garde le rideau. Elle refuse de foncer, dit d'accord, enfile seule. Merci vécu. La rouge file dans la dentelle. L'éclat de couvercle tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La boîte à couture sent la cire. Le couvercle est lisse, un peu chaud. Une pelote de laine dort dans un coin. La laine est grise, un peu rêche. Dedans, des perles de bois dorment. Brunes. Beiges. Une rouge, toute ronde. Le rideau de dentelle fait des trous de lumière. Un carré de soleil touche le fil. Tu as senti la cire, Nina ? Oui, papa. Ça sent le bois aussi. On reste au sec, d'accord ? D'accord, maman. Je fais un collier. Pour toi. Pour moi ? Oui. En ce moment, Nina prend un fil. Le fil est un peu raide. Victorino est près de la fenêtre. Il tient un pli du rideau. Tu viens ? Je regarde. Nina accepte. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Nina enfile une perle brune. Ça fait un petit glissement. Le fil tremble un peu. Plus tard ? Plus tard. D'accord. Tu as accepté, Nina ? Oui, papa. Regarder, c'est une réponse. La perle rouge roule. Elle se cache dans la dentelle. Tu as vu le trou de lumière ? La perle est dedans.</t>
+          <t>Un carré de soleil perce le rideau de dentelle. Des trous de lumière tombent sur le plancher. La cire sent chaud, sous le rayon. Ça sent bon, maman. C'est la boîte à couture. La boîte à couture attend près du canapé. Le couvercle est lisse, un peu chaud. Sur le couvercle, un éclat de couvercle brille. Il brille, papa ! Tu le vois, Nina ? Oui, sur le couvercle. Une pelote de laine dort dans un coin. La pelote est grise, un peu rêche. Elle reste dans la boîte ? Oui, maman. Dedans, des perles dorment. Brunes. Beiges. Une rouge, toute ronde. La rouge est pour toi. Pour moi ? Oui. Je fais un collier, maintenant ! Tu prends le fil ? Oui, papa. Papa glisse un fil vers elle. Le fil est un peu raide. Le coin de la dentelle est clair, sous le rayon. En ce moment, Nina tire le fil trop vite. Le fil se tord entre les doigts. Oh. Victorino est près de la fenêtre. Il tient un pli du rideau. La dentelle chatouille ses doigts. Tu viens ? Victorino ne dit rien. Il garde le pli, sans bouger. Prends le fil ! Nina pousse le fil vers sa main. La main de Victorino reste sur le rideau. Le fil tombe sur le plancher. Une perle brune glisse, presque. Ça ne veut pas. Le sourire de Nina s'en va. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de couvercle tremble, puis tient. Ses épaules tombent un peu, lourdes. Tu veux qu'il vienne ? Oui, papa. Papa se baisse à sa hauteur. Le fil est là, près du pied. Je le reprends. Nina ramasse le fil, un peu froissé. Je regarde. Maintenant ? Victorino secoue la tête, très peu. Tu l'as entendu, Nina ? Il regarde.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La boîte à couture sent la cire. Le couvercle est lisse, un peu chaud. Une pelote de laine dort dans un coin. La laine est grise, un peu rêche. Dedans, des perles de bois dorment. Brunes. Beiges. Une rouge, toute ronde. Le rideau de dentelle fait des trous de lumière. Un carré de soleil touche le fil. Tu as senti la cire, Nina ? Oui, papa. Ça sent le bois aussi. On reste au sec, d'accord ? D'accord, maman. Je fais un collier. Pour toi. Pour moi ? Oui. En ce moment, Nina prend un fil. Le fil est un peu raide. Victorino est près de la fenêtre. Il tient un pli du rideau. Tu viens ? Je regarde. Nina accepte. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Nina enfile une perle brune. Ça fait un petit glissement. Le fil tremble un peu. Plus tard ? Plus tard. D'accord. Tu as accepté, Nina ? Oui, papa. Regarder, c'est une réponse. La perle rouge roule. Elle se cache dans la dentelle. Tu as vu le trou de lumière ? La perle est dedans.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un carré de soleil perce le rideau de dentelle. Des trous de lumière tombent sur le plancher. La cire sent chaud, sous le rayon. Ça sent bon, maman. C'est la boîte à couture. La boîte à couture attend près du canapé. Le couvercle est lisse, un peu chaud. Sur le couvercle, un &lt;emphasis level="moderate"&gt;éclat de couvercle&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, Nina ? Oui, sur le couvercle. Une pelote de laine dort dans un coin. La pelote est grise, un peu rêche. Elle reste dans la boîte ? Oui, maman. Dedans, des perles dorment. Brunes. Beiges. Une rouge, toute ronde. La rouge est pour toi. Pour moi ? Oui. Je fais un collier, maintenant ! Tu prends le fil ? Oui, papa. Papa glisse un fil vers elle. Le fil est un peu raide. Le coin de la dentelle est clair, sous le rayon. En ce moment, Nina tire le fil trop vite. Le fil se tord entre les doigts. Oh. Victorino est près de la fenêtre. Il tient un pli du rideau. La dentelle chatouille ses doigts. Tu viens ? Victorino ne dit rien. Il garde le pli, sans bouger. Prends le fil ! Nina pousse le fil vers sa main. La main de Victorino reste sur le rideau. Le fil tombe sur le plancher. Une perle brune glisse, presque. Ça ne veut pas. Le sourire de Nina s'en va. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de couvercle tremble, puis tient. Ses épaules tombent un peu, lourdes. Tu veux qu'il vienne ? Oui, papa. Papa se baisse à sa hauteur. Le fil est là, près du pied. Je le reprends. Nina ramasse le fil, un peu froissé. Je regarde. Maintenant ? Victorino secoue la tête, très peu. Tu l'as entendu, Nina ? Il regarde.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ninon est dans le salon avec maman. Octave est près du canapé. Ninon va &lt;emphasis&gt;proposer&lt;/emphasis&gt; les cubes. Elle dit : tu viens ? Octave dit : je regarde. Ninon accepte. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Ninon construit. Octave regarde. Ninon propose encore, tout doux : plus tard ? Octave dit : plus tard. Ninon dit : d'accord. [pause]</t>
+          <t>Un carré de soleil perce le rideau de dentelle. Des trous de lumière tombent sur le plancher. La cire sent chaud, sous le rayon. Ça sent bon, maman. C'est la boîte à couture. La boîte à couture attend près du canapé. Le couvercle est lisse, un peu chaud. Sur le couvercle, un &lt;emphasis&gt;éclat de couvercle&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, Nina ? Oui, sur le couvercle. Une pelote de laine dort dans un coin. La pelote est grise, un peu rêche. Elle reste dans la boîte ? Oui, maman. Dedans, des perles dorment. Brunes. Beiges. Une rouge, toute ronde. La rouge est pour toi. Pour moi ? Oui. Je fais un collier, maintenant ! Tu prends le fil ? Oui, papa. Papa glisse un fil vers elle. Le fil est un peu raide. Le coin de la dentelle est clair, sous le rayon. En ce moment, Nina tire le fil trop vite. Le fil se tord entre les doigts. Oh. Victorino est près de la fenêtre. Il tient un pli du rideau. La dentelle chatouille ses doigts. Tu viens ? Victorino ne dit rien. Il garde le pli, sans bouger. Prends le fil ! Nina pousse le fil vers sa main. La main de Victorino reste sur le rideau. Le fil tombe sur le plancher. Une perle brune glisse, presque. Ça ne veut pas. Le sourire de Nina s'en va. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'éclat de couvercle tremble, puis tient. Ses épaules tombent un peu, lourdes. Tu veux qu'il vienne ? Oui, papa. Papa se baisse à sa hauteur. Le fil est là, près du pied. Je le reprends. Nina ramasse le fil, un peu froissé. Je regarde. Maintenant ? Victorino secoue la tête, très peu. Tu l'as entendu, Nina ? Il regarde. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat de couvercle</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,54 +1326,71 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_collier_et_victorino_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La boîte à couture sent la cire.
+          <t>narrateur|Un carré de soleil perce le rideau de dentelle.
+narrateur|Des trous de lumière tombent sur le plancher.
+narrateur|La cire sent chaud, sous le rayon.
+enfant-f|Ça sent bon, maman.
+maman|C'est la boîte à couture.
+narrateur|La boîte à couture attend près du canapé.
 narrateur|Le couvercle est lisse, un peu chaud.
+narrateur|Sur le couvercle, un éclat de couvercle brille.
+enfant-f|Il brille, papa !
+papa|Tu le vois, Nina ?
+enfant-f|Oui, sur le couvercle.
 narrateur|Une pelote de laine dort dans un coin.
-narrateur|La laine est grise, un peu rêche.
-narrateur|Dedans, des perles de bois dorment.
+narrateur|La pelote est grise, un peu rêche.
+maman|Elle reste dans la boîte ?
+enfant-f|Oui, maman.
+narrateur|Dedans, des perles dorment.
 narrateur|Brunes.
 narrateur|Beiges.
 narrateur|Une rouge, toute ronde.
-narrateur|Le rideau de dentelle fait des trous de lumière.
-narrateur|Un carré de soleil touche le fil.
-papa|Tu as senti la cire, Nina ?
-enfant-f|Oui, papa.
-enfant-f|Ça sent le bois aussi.
-maman|On reste au sec, d'accord ?
-enfant-f|D'accord, maman.
-enfant-f|Je fais un collier.
-enfant-f|Pour toi.
+enfant-f|La rouge est pour toi.
 maman|Pour moi ?
 enfant-f|Oui.
-narrateur|En ce moment, Nina prend un fil.
+enfant-f|Je fais un collier, maintenant !
+papa|Tu prends le fil ?
+enfant-f|Oui, papa.
+narrateur|Papa glisse un fil vers elle.
 narrateur|Le fil est un peu raide.
+narrateur|Le coin de la dentelle est clair, sous le rayon.
+narrateur|En ce moment, Nina tire le fil trop vite.
+narrateur|Le fil se tord entre les doigts.
+enfant-f|Oh.
 narrateur|Victorino est près de la fenêtre.
 narrateur|Il tient un pli du rideau.
+narrateur|La dentelle chatouille ses doigts.
 enfant-f|Tu viens ?
+narrateur|Victorino ne dit rien.
+narrateur|Il garde le pli, sans bouger.
+enfant-f|Prends le fil !
+narrateur|Nina pousse le fil vers sa main.
+narrateur|La main de Victorino reste sur le rideau.
+narrateur|Le fil tombe sur le plancher.
+narrateur|Une perle brune glisse, presque.
+enfant-f|Ça ne veut pas.
+narrateur|Le sourire de Nina s'en va.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|L'éclat de couvercle tremble, puis tient.
+narrateur|Ses épaules tombent un peu, lourdes.
+papa|Tu veux qu'il vienne ?
+enfant-f|Oui, papa.
+narrateur|Papa se baisse à sa hauteur.
+maman|Le fil est là, près du pied.
+enfant-f|Je le reprends.
+narrateur|Nina ramasse le fil, un peu froissé.
 copain|Je regarde.
-narrateur|Nina accepte.
-maman|On peut proposer.
-maman|On peut accepter plusieurs réponses.
-papa|Oui.
-papa|Non.
-papa|Regarder.
-papa|Plus tard.
-narrateur|Nina enfile une perle brune.
-narrateur|Ça fait un petit glissement.
-narrateur|Le fil tremble un peu.
-enfant-f|Plus tard ?
-copain|Plus tard.
-enfant-f|D'accord.
-papa|Tu as accepté, Nina ?
-enfant-f|Oui, papa.
-maman|Regarder, c'est une réponse.
-narrateur|La perle rouge roule.
-narrateur|Elle se cache dans la dentelle.
-papa|Tu as vu le trou de lumière ?
-enfant-f|La perle est dedans.</t>
+enfant-f|Maintenant ?
+narrateur|Victorino secoue la tête, très peu.
+papa|Tu l'as entendu, Nina ?
+enfant-f|Il regarde.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1410,12 +1427,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina invite Victorino. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina &lt;emphasis level="moderate"&gt;invite&lt;/emphasis&gt; Victorino. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ninon invite Octave. Que fait-elle si Octave dit non ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina &lt;emphasis&gt;invite&lt;/emphasis&gt; Victorino. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1478,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1489,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>invite</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1546,17 +1567,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_invite_puis_elle_prend_sa_reponse; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a su proposer. Elle a su accepter plusieurs réponses. Victorino a dit regarder, puis plus tard. Oui. Tout ça va. J'ai dit d'accord. Nina cherche dans la dentelle. Le fil du rideau chatouille un peu. Ses doigts trouvent la perle rouge. Te voilà. Bravo. Tu as retrouvé la perle. Tu veux la rouge ? Non. D'accord. Plusieurs réponses sont possibles. Nina enfile la rouge. Le collier s'allonge. Les perles tapent l'une contre l'autre. Victorino s'assoit sur ses talons. Il regarde encore. Tu as proposé tout doux ? Oui, maman.</t>
+          <t>Nina se penche trop vite vers Victorino. Viens, maintenant ! Victorino reste près du rideau. Plus tard. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle regarde le pli du rideau. Tu le vois, près de la fenêtre ? Oui. Victorino garde le silence, un moment. D'accord. Nina reprend le fil, sans se presser. Elle enfile une perle brune. Ça fait un petit glissement. Tu veux la beige ? Victorino ne tend pas la main. Je regarde. D'accord. Nina enfile la beige, toute seule. Les perles tapent l'une contre l'autre. Victorino s'assoit sur ses talons. Il regarde le fil, sans parler. Sur le couvercle, l'éclat de couvercle brille. Il est là. Sur le couvercle ? Oui, papa. Merci, Nina. Maman a entendu toute la phrase. Le ventre de Nina se desserre. Tu as les mains prêtes ? Un peu, papa. Le collier s'allonge, lentement. La rouge attend ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a su proposer. Elle a su accepter plusieurs réponses. Victorino a dit regarder, puis plus tard. Oui. Tout ça va. J'ai dit d'accord. Nina cherche dans la dentelle. Le fil du rideau chatouille un peu. Ses doigts trouvent la perle rouge. Te voilà. Bravo. Tu as retrouvé la perle. Tu veux la rouge ? Non. D'accord. Plusieurs réponses sont possibles. Nina enfile la rouge. Le collier s'allonge. Les perles tapent l'une contre l'autre. Victorino s'assoit sur ses talons. Il regarde encore. Tu as proposé tout doux ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina se penche trop vite vers Victorino. Viens, maintenant ! Victorino reste près du rideau. Plus tard. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle regarde le pli du rideau. Tu le vois, près de la fenêtre ? Oui. Victorino garde le silence, un moment. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Nina reprend le fil, sans se presser. Elle enfile une perle brune. Ça fait un petit glissement. Tu veux la beige ? Victorino ne tend pas la main. Je regarde. D'accord. Nina enfile la beige, toute seule. Les perles tapent l'une contre l'autre. Victorino s'assoit sur ses talons. Il regarde le fil, sans parler. Sur le couvercle, l'éclat de couvercle brille. Il est là. Sur le couvercle ? Oui, papa. Merci, Nina. Maman a entendu toute la phrase. Le ventre de Nina se desserre. Tu as les mains prêtes ? Un peu, papa. Le collier s'allonge, lentement. La rouge attend ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ninon a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Elle a su accepter plusieurs réponses. [pause]</t>
+          <t>Nina se penche trop vite vers Victorino. Viens, maintenant ! Victorino reste près du rideau. Plus tard. Oh. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Elle referme la bouche, un instant. Elle regarde le pli du rideau. Tu le vois, près de la fenêtre ? Oui. Victorino garde le silence, un moment. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Nina reprend le fil, sans se presser. Elle enfile une perle brune. Ça fait un petit glissement. Tu veux la beige ? Victorino ne tend pas la main. Je regarde. D'accord. Nina enfile la beige, toute seule. Les perles tapent l'une contre l'autre. Victorino s'assoit sur ses talons. Il regarde le fil, sans parler. Sur le couvercle, l'éclat de couvercle brille. Il est là. Sur le couvercle ? Oui, papa. Merci, Nina. Maman a entendu toute la phrase. Le ventre de Nina se desserre. Tu as les mains prêtes ? Un peu, papa. Le collier s'allonge, lentement. La rouge attend ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1667,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1675,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,30 +1701,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1733,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1728,33 +1749,46 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_dit_daccord_et_enfile_seule; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a su proposer.
-narrateur|Elle a su accepter plusieurs réponses.
-papa|Victorino a dit regarder, puis plus tard.
-maman|Oui.
-maman|Tout ça va.
-enfant-f|J'ai dit d'accord.
-narrateur|Nina cherche dans la dentelle.
-narrateur|Le fil du rideau chatouille un peu.
-narrateur|Ses doigts trouvent la perle rouge.
-enfant-f|Te voilà.
-papa|Bravo.
-papa|Tu as retrouvé la perle.
-enfant-f|Tu veux la rouge ?
-copain|Non.
+          <t>narrateur|Nina se penche trop vite vers Victorino.
+enfant-f|Viens, maintenant !
+narrateur|Victorino reste près du rideau.
+copain|Plus tard.
+enfant-f|Oh.
+narrateur|Le sourire de Nina ne revient pas.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Elle referme la bouche, un instant.
+narrateur|Elle regarde le pli du rideau.
+papa|Tu le vois, près de la fenêtre ?
+enfant-f|Oui.
+narrateur|Victorino garde le silence, un moment.
 enfant-f|D'accord.
-maman|Plusieurs réponses sont possibles.
-narrateur|Nina enfile la rouge.
-narrateur|Le collier s'allonge.
+narrateur|Nina reprend le fil, sans se presser.
+narrateur|Elle enfile une perle brune.
+narrateur|Ça fait un petit glissement.
+enfant-f|Tu veux la beige ?
+narrateur|Victorino ne tend pas la main.
+copain|Je regarde.
+enfant-f|D'accord.
+narrateur|Nina enfile la beige, toute seule.
 narrateur|Les perles tapent l'une contre l'autre.
 narrateur|Victorino s'assoit sur ses talons.
-narrateur|Il regarde encore.
-maman|Tu as proposé tout doux ?
+narrateur|Il regarde le fil, sans parler.
+narrateur|Sur le couvercle, l'éclat de couvercle brille.
+enfant-f|Il est là.
+papa|Sur le couvercle ?
+enfant-f|Oui, papa.
+maman|Merci, Nina.
+narrateur|Maman a entendu toute la phrase.
+narrateur|Le ventre de Nina se desserre.
+papa|Tu as les mains prêtes ?
+enfant-f|Un peu, papa.
+narrateur|Le collier s'allonge, lentement.
+maman|La rouge attend ?
 enfant-f|Oui, maman.</t>
         </is>
       </c>
@@ -1787,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On noue le fil ? Oui. Papa tient le nœud. Nina tire, tout doux. Le collier est fermé. Tu as fini le collier, Nina ? Oui, papa. Maman baisse un peu la tête. Nina passe le collier. Les perles tapent, tout doux. La perle rouge se met au milieu. Il est beau. Merci, Nina. Victorino a regardé. Oui. C'est une réponse. La lumière perce encore la dentelle. La perle rouge brille au milieu. Maman touche le bois, tout doux.</t>
+          <t>Nina veut la perle rouge, d'un coup. Regarde, la rouge ! Elle tend la perle trop vite. Tu veux la rouge ? Non. Nina veut la poser dans sa main. La perle rouge file entre les doigts. Ça tombe ! La rouge se cache dans la dentelle. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la boîte à couture. Elle écoute le salon, un instant. La poussière danse dans le rayon. Sur le couvercle, l'éclat de couvercle revient. Comme ce matin ? Tu le vois, toi ? Oui, sur le couvercle. Nina cherche dans la dentelle. Le fil du rideau chatouille un peu. Ses doigts trouvent la perle rouge. Te voilà. Je la mets, moi. Elle enfile la rouge, sans se presser. Au milieu ? Oui, papa. Le collier s'allonge ? Oui, maman. Victorino reste sur ses talons. Il regarde la rouge, sans la prendre. Elle est lisse.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On noue le fil ? Oui. Papa tient le nœud. Nina tire, tout doux. Le collier est fermé. Tu as fini le collier, Nina ? Oui, papa. Maman baisse un peu la tête. Nina passe le collier. Les perles tapent, tout doux. La perle rouge se met au milieu. Il est beau. Merci, Nina. Victorino a regardé. Oui. C'est une réponse. La lumière perce encore la dentelle. La perle rouge brille au milieu. Maman touche le bois, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina veut la perle rouge, d'un coup. Regarde, la rouge ! Elle tend la perle trop vite. Tu veux la rouge ? Non. Nina veut la poser dans sa main. La perle rouge file entre les doigts. Ça tombe ! La rouge se cache dans la dentelle. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la boîte à couture. Elle écoute le salon, un instant. La poussière danse dans le rayon. Sur le couvercle, l'&lt;emphasis level="moderate"&gt;éclat de couvercle&lt;/emphasis&gt; revient. Comme ce matin ? Tu le vois, toi ? Oui, sur le couvercle. Nina cherche dans la dentelle. Le fil du rideau chatouille un peu. Ses doigts trouvent la perle rouge. Te voilà. Je la mets, moi. Elle enfile la rouge, sans se presser. Au milieu ? Oui, papa. Le collier s'allonge ? Oui, maman. Victorino reste sur ses talons. Il regarde la rouge, sans la prendre. Elle est lisse.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range un cube. Ninon donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Nina veut la perle rouge, d'un coup. Regarde, la rouge ! Elle tend la perle trop vite. Tu veux la rouge ? Non. Nina veut la poser dans sa main. La perle rouge file entre les doigts. Ça tombe ! La rouge se cache dans la dentelle. Nina veut foncer, d'un coup. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la boîte à couture. Elle écoute le salon, un instant. La poussière danse dans le rayon. Sur le couvercle, l'&lt;emphasis&gt;éclat de couvercle&lt;/emphasis&gt; revient. Comme ce matin ? Tu le vois, toi ? Oui, sur le couvercle. Nina cherche dans la dentelle. Le fil du rideau chatouille un peu. Ses doigts trouvent la perle rouge. Te voilà. Je la mets, moi. Elle enfile la rouge, sans se presser. Au milieu ? Oui, papa. Le collier s'allonge ? Oui, maman. Victorino reste sur ses talons. Il regarde la rouge, sans la prendre. Elle est lisse.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1844,7 +1878,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1852,22 +1886,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1878,30 +1916,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de couvercle</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1910,42 +1948,61 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On noue le fil ?
-enfant-f|Oui.
-narrateur|Papa tient le nœud.
-narrateur|Nina tire, tout doux.
-narrateur|Le collier est fermé.
-papa|Tu as fini le collier, Nina ?
+          <t>narrateur|Nina veut la perle rouge, d'un coup.
+enfant-f|Regarde, la rouge !
+narrateur|Elle tend la perle trop vite.
+enfant-f|Tu veux la rouge ?
+copain|Non.
+narrateur|Nina veut la poser dans sa main.
+narrateur|La perle rouge file entre les doigts.
+enfant-f|Ça tombe !
+narrateur|La rouge se cache dans la dentelle.
+narrateur|Nina veut foncer, d'un coup.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde la boîte à couture.
+narrateur|Elle écoute le salon, un instant.
+narrateur|La poussière danse dans le rayon.
+narrateur|Sur le couvercle, l'éclat de couvercle revient.
+enfant-f|Comme ce matin ?
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le couvercle.
+narrateur|Nina cherche dans la dentelle.
+narrateur|Le fil du rideau chatouille un peu.
+narrateur|Ses doigts trouvent la perle rouge.
+enfant-f|Te voilà.
+enfant-f|Je la mets, moi.
+narrateur|Elle enfile la rouge, sans se presser.
+papa|Au milieu ?
 enfant-f|Oui, papa.
-narrateur|Maman baisse un peu la tête.
-narrateur|Nina passe le collier.
-narrateur|Les perles tapent, tout doux.
-narrateur|La perle rouge se met au milieu.
-maman|Il est beau.
-maman|Merci, Nina.
-enfant-f|Victorino a regardé.
-papa|Oui.
-papa|C'est une réponse.
-narrateur|La lumière perce encore la dentelle.
-narrateur|La perle rouge brille au milieu.
-narrateur|Maman touche le bois, tout doux.</t>
+maman|Le collier s'allonge ?
+enfant-f|Oui, maman.
+narrateur|Victorino reste sur ses talons.
+narrateur|Il regarde la rouge, sans la prendre.
+enfant-f|Elle est lisse.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1977,17 +2034,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le collier repose sur maman. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. La boîte à couture sent encore la cire.</t>
+          <t>On noue le fil ? Oui. Papa tient le nœud. Nina tire, sans se presser. Le collier est fermé. Le collier est pour maman ? Oui, papa. Maman baisse un peu la tête. Nina passe le collier. Les perles tapent contre le cou. La perle rouge se met au milieu. Il est beau. Victorino a regardé. Tu le vois, sur maman ? Oui, papa. La lumière perce la dentelle. La boîte à couture sent la cire. L'éclat est là, papa. Tu le vois sur le couvercle ? Oui, papa. On est bien, ici. Nina pose la joue près du couvercle. Le couvercle est lisse, un peu chaud. C'est chaud. Victorino lâche le pli du rideau. L'éclat de couvercle tient sur le couvercle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le collier repose sur maman. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. La boîte à couture sent encore la cire.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;On noue le fil ? Oui. Papa tient le nœud. Nina tire, sans se presser. Le collier est fermé. Le collier est pour maman ? Oui, papa. Maman baisse un peu la tête. Nina passe le collier. Les perles tapent contre le cou. La perle rouge se met au milieu. Il est beau. Victorino a regardé. Tu le vois, sur maman ? Oui, papa. La lumière perce la dentelle. La boîte à couture sent la cire. L'éclat est là, papa. Tu le vois sur le couvercle ? Oui, papa. On est bien, ici. Nina pose la joue près du couvercle. Le couvercle est lisse, un peu chaud. C'est chaud. Victorino lâche le pli du rideau. L'&lt;emphasis level="moderate"&gt;éclat de couvercle&lt;/emphasis&gt; tient sur le couvercle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;On noue le fil ? Oui. Papa tient le nœud. Nina tire, sans se presser. Le collier est fermé. Le collier est pour maman ? Oui, papa. Maman baisse un peu la tête. Nina passe le collier. Les perles tapent contre le cou. La perle rouge se met au milieu. Il est beau. Victorino a regardé. Tu le vois, sur maman ? Oui, papa. La lumière perce la dentelle. La boîte à couture sent la cire. L'éclat est là, papa. Tu le vois sur le couvercle ? Oui, papa. On est bien, ici. Nina pose la joue près du couvercle. Le couvercle est lisse, un peu chaud. C'est chaud. Victorino lâche le pli du rideau. L'&lt;emphasis&gt;éclat de couvercle&lt;/emphasis&gt; tient sur le couvercle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2034,18 +2091,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2054,12 +2111,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2068,17 +2125,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de couvercle</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2087,11 +2148,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2100,29 +2161,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_couvercle; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le collier repose sur maman.
-enfant-f|J'ai proposé.
-enfant-f|J'ai accepté.
-maman|Plusieurs réponses sont possibles.
-papa|Oui.
-narrateur|La boîte à couture sent encore la cire.</t>
+          <t>maman|On noue le fil ?
+enfant-f|Oui.
+narrateur|Papa tient le nœud.
+narrateur|Nina tire, sans se presser.
+narrateur|Le collier est fermé.
+papa|Le collier est pour maman ?
+enfant-f|Oui, papa.
+narrateur|Maman baisse un peu la tête.
+narrateur|Nina passe le collier.
+narrateur|Les perles tapent contre le cou.
+narrateur|La perle rouge se met au milieu.
+maman|Il est beau.
+enfant-f|Victorino a regardé.
+papa|Tu le vois, sur maman ?
+enfant-f|Oui, papa.
+narrateur|La lumière perce la dentelle.
+narrateur|La boîte à couture sent la cire.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur le couvercle ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|Nina pose la joue près du couvercle.
+narrateur|Le couvercle est lisse, un peu chaud.
+enfant-f|C'est chaud.
+narrateur|Victorino lâche le pli du rideau.
+narrateur|L'éclat de couvercle tient sur le couvercle.</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2221,6 +2306,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>